<commit_message>
Add tag to NON PHPL upload
</commit_message>
<xml_diff>
--- a/public/samples/Sample_NonPHPL_Upload.xlsx
+++ b/public/samples/Sample_NonPHPL_Upload.xlsx
@@ -413,30 +413,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Patient Name</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Mobile Number</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>UMR Number</t>
+          <t>UMR</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -447,6 +448,11 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>Discount %</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Tag</t>
         </is>
       </c>
     </row>
@@ -461,15 +467,22 @@
           <t>9876543210</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UMR001</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>NON PHPL</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>20</t>
+      <c r="E2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>DAILY</t>
         </is>
       </c>
     </row>
@@ -484,36 +497,16 @@
           <t>9123456789</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>UMR001</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>NON PHPL</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>9988776655</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NON PHPL</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>